<commit_message>
feat: upsert target produksi + kolom WP&B/RKAP, samakan SP dan seeding dengan master, tambah setup_db
</commit_message>
<xml_diff>
--- a/frontend/public/templates/Template - Produksi.xlsx
+++ b/frontend/public/templates/Template - Produksi.xlsx
@@ -8752,12 +8752,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <cols>
     <col width="12.3984375" customWidth="1" min="1" max="1"/>
     <col width="14.8984375" customWidth="1" min="2" max="2"/>
-    <col width="14.8984375" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8767,7 +8769,8 @@
         </is>
       </c>
       <c r="C1" s="4" t="n"/>
-      <c r="D1" s="5" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8782,7 +8785,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KONDENSAT</t>
+          <t>GAS WP&amp;B</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KONDENSAT RKAP</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>KONDENSAT WP&amp;B</t>
         </is>
       </c>
     </row>
@@ -8793,6 +8806,15 @@
       <c r="B3" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C3" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D3" t="n">
+        <v>738</v>
+      </c>
+      <c r="E3" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -8801,6 +8823,15 @@
       <c r="B4" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C4" t="n">
+        <v>85.12714286000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>738</v>
+      </c>
+      <c r="E4" t="n">
+        <v>619.71</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -8809,6 +8840,15 @@
       <c r="B5" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C5" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D5" t="n">
+        <v>738</v>
+      </c>
+      <c r="E5" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -8817,6 +8857,15 @@
       <c r="B6" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C6" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D6" t="n">
+        <v>738</v>
+      </c>
+      <c r="E6" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -8825,6 +8874,15 @@
       <c r="B7" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C7" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D7" t="n">
+        <v>738</v>
+      </c>
+      <c r="E7" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -8833,6 +8891,15 @@
       <c r="B8" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C8" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D8" t="n">
+        <v>738</v>
+      </c>
+      <c r="E8" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -8841,6 +8908,15 @@
       <c r="B9" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C9" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D9" t="n">
+        <v>738</v>
+      </c>
+      <c r="E9" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -8849,6 +8925,15 @@
       <c r="B10" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C10" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D10" t="n">
+        <v>738</v>
+      </c>
+      <c r="E10" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -8857,6 +8942,15 @@
       <c r="B11" t="n">
         <v>94.40000000000002</v>
       </c>
+      <c r="C11" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D11" t="n">
+        <v>738</v>
+      </c>
+      <c r="E11" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -8865,6 +8959,15 @@
       <c r="B12" t="n">
         <v>93.59999999999999</v>
       </c>
+      <c r="C12" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D12" t="n">
+        <v>738</v>
+      </c>
+      <c r="E12" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -8873,6 +8976,15 @@
       <c r="B13" t="n">
         <v>93.59999999999999</v>
       </c>
+      <c r="C13" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D13" t="n">
+        <v>738</v>
+      </c>
+      <c r="E13" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -8881,10 +8993,19 @@
       <c r="B14" t="n">
         <v>93.59999999999999</v>
       </c>
+      <c r="C14" t="n">
+        <v>93.47</v>
+      </c>
+      <c r="D14" t="n">
+        <v>738</v>
+      </c>
+      <c r="E14" t="n">
+        <v>724</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>